<commit_message>
Parse multiline blocks and write CSV output
Improve parsing of multi-line, space-aligned blocks and add CSV output. TxtParser.parseMultiLineGroupedBlock now detects dynamic headers from the input line, computes absolute column boundaries, extracts column substrings safely (getSafeSubstring), and preserves header rows between @101 blocks. DiagnoseBlocks was updated to call the parser, log progress, and write the parsed rows to FTX/result QV.csv. Added expected and result CSV fixtures (FTX/Expected QV.csv, FTX/result QV.csv). Also includes unrelated build/report binary updates and an updated problems-report.html snapshot.
</commit_message>
<xml_diff>
--- a/FTX/output888 - outcome 3sets.xlsx
+++ b/FTX/output888 - outcome 3sets.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="74">
   <si>
     <t>Element</t>
   </si>
@@ -197,6 +197,12 @@
     <t>Up Tol.</t>
   </si>
   <si>
+    <t>Up Tol. (1)</t>
+  </si>
+  <si>
+    <t>Up Tol. (2)</t>
+  </si>
+  <si>
     <t>0.0200</t>
   </si>
   <si>
@@ -206,10 +212,22 @@
     <t>Low Tol.</t>
   </si>
   <si>
+    <t>Low Tol. (1)</t>
+  </si>
+  <si>
+    <t>Low Tol. (2)</t>
+  </si>
+  <si>
     <t>-0.0200</t>
   </si>
   <si>
     <t>Pass/Fail</t>
+  </si>
+  <si>
+    <t>Pass/Fail (1)</t>
+  </si>
+  <si>
+    <t>Pass/Fail (2)</t>
   </si>
   <si>
     <t>PASS</t>
@@ -260,7 +278,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:P17"/>
+  <dimension ref="A1:M17"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -280,37 +298,28 @@
         <v>60</v>
       </c>
       <c r="F1" t="s" s="0">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="G1" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="H1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="I1" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="J1" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="K1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="L1" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="M1" t="s">
-        <v>65</v>
-      </c>
-      <c r="N1" t="s">
-        <v>60</v>
-      </c>
-      <c r="O1" t="s">
-        <v>63</v>
-      </c>
-      <c r="P1" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
     </row>
     <row r="2">
@@ -327,31 +336,31 @@
         <v>45</v>
       </c>
       <c r="E2" t="s" s="0">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F2" t="s" s="0">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="G2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="J2" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="K2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="L2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="M2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3">
@@ -368,31 +377,31 @@
         <v>46</v>
       </c>
       <c r="E3" t="s" s="0">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F3" t="s" s="0">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G3" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="I3" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="J3" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="K3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="L3" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="M3" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4">
@@ -409,31 +418,31 @@
         <v>47</v>
       </c>
       <c r="E4" t="s" s="0">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F4" t="s" s="0">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G4" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H4" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="I4" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="J4" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="K4" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="L4" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="M4" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5">
@@ -450,31 +459,31 @@
         <v>48</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F5" t="s" s="0">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G5" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H5" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="I5" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="J5" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="K5" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="L5" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="M5" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6">
@@ -491,31 +500,31 @@
         <v>49</v>
       </c>
       <c r="E6" t="s" s="0">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F6" t="s" s="0">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G6" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H6" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="I6" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="J6" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="K6" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="L6" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="M6" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7">
@@ -532,31 +541,31 @@
         <v>50</v>
       </c>
       <c r="E7" t="s" s="0">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F7" t="s" s="0">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G7" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="H7" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="I7" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="J7" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="K7" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="L7" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="M7" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
     </row>
     <row r="8">
@@ -573,31 +582,31 @@
         <v>51</v>
       </c>
       <c r="E8" t="s" s="0">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F8" t="s" s="0">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G8" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="H8" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="I8" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="J8" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="K8" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="L8" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="M8" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
     </row>
     <row r="9">
@@ -614,31 +623,31 @@
         <v>52</v>
       </c>
       <c r="E9" t="s" s="0">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F9" t="s" s="0">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G9" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H9" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I9" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="J9" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="K9" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="L9" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="M9" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="10">
@@ -655,31 +664,31 @@
         <v>53</v>
       </c>
       <c r="E10" t="s" s="0">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F10" t="s" s="0">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G10" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H10" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I10" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="J10" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="K10" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="L10" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="M10" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="11">
@@ -696,31 +705,31 @@
         <v>54</v>
       </c>
       <c r="E11" t="s" s="0">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F11" t="s" s="0">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G11" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I11" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="J11" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="K11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="L11" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="M11" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="12">
@@ -737,31 +746,31 @@
         <v>55</v>
       </c>
       <c r="E12" t="s" s="0">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F12" t="s" s="0">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G12" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I12" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="J12" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="K12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="L12" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="M12" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="13">
@@ -778,31 +787,31 @@
         <v>56</v>
       </c>
       <c r="E13" t="s" s="0">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F13" t="s" s="0">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G13" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H13" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I13" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="J13" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="K13" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="L13" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="M13" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="14">
@@ -819,31 +828,31 @@
         <v>57</v>
       </c>
       <c r="E14" t="s" s="0">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F14" t="s" s="0">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G14" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H14" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I14" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="J14" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="K14" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="L14" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="M14" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="15">
@@ -860,31 +869,31 @@
         <v>58</v>
       </c>
       <c r="E15" t="s" s="0">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F15" t="s" s="0">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G15" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H15" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I15" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="J15" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="K15" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="L15" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="M15" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="16">
@@ -901,31 +910,31 @@
         <v>59</v>
       </c>
       <c r="E16" t="s" s="0">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F16" t="s" s="0">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G16" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H16" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I16" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="J16" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="K16" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="L16" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="M16" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="17">
@@ -942,31 +951,31 @@
         <v>33</v>
       </c>
       <c r="E17" t="s" s="0">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F17" t="s" s="0">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G17" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="H17" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I17" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="J17" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="K17" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="L17" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="M17" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>